<commit_message>
Update data dictionary with derived columns and leakage notes
</commit_message>
<xml_diff>
--- a/reports/Data Dictionary.xlsx
+++ b/reports/Data Dictionary.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\projects\bank-marketing-segmentation\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F1B990B0-2489-4E7B-97A5-1CD3188641AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35A5C3B0-F777-4609-986E-2AD7AF3AA7DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{55FA88CE-5E89-4531-8B8B-8103CBAE7C2D}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="177">
   <si>
     <t>Data Dictionary: Bank Marketing Dataset</t>
   </si>
@@ -275,9 +275,6 @@
     <t>No. It is known only after the call ends.</t>
   </si>
   <si>
-    <t>Excluded from predictive modelling because it causes target leakage.</t>
-  </si>
-  <si>
     <t>campaign</t>
   </si>
   <si>
@@ -290,9 +287,6 @@
     <t>No, not in its final form at the initial decision point.</t>
   </si>
   <si>
-    <t>Excluded from model inputs; used for retrospective contact-efficiency analysis.</t>
-  </si>
-  <si>
     <t>contact_band</t>
   </si>
   <si>
@@ -543,6 +537,39 @@
   </si>
   <si>
     <t>The following rules will guide the data pipeline:                                                                                                                                                                                                                                                                 1. Exclude duration because it is only known after a call and can leak information about the outcome.                                                                                                                                                                                               2. Exclude campaign and contact_band from initial prediction. Both describe current-campaign contact effort and are intended for retrospective evaluation.                                     3. Assess contact, month, and day_of_week carefully. Their availability depends on the decision being modelled. Channel and timing information should only be used if it would genuinely be available at the point of prediction.                                                                                                                                                                                              4. Validate the economic indicators. Confirm that each value was available at the decision date and determine whether the model relies too heavily on historical economic conditions.                                                                                                                                                                                                                                                             5. Evaluate fairness across age, marital status and education. The dataset has no gender column, so gender fairness cannot be assessed directly.                                                                    6. Protect the data. Keep confidential data out of the public repository and document the source, licence, access date and file checksum.</t>
+  </si>
+  <si>
+    <t>Excluded from predictive modelling because it causes target leakage. Excluded from model inputs (known only after the call ends). Kept in the full cleaned table; removed from bank_marketing_model_inputs.csv by select_model_inputs().</t>
+  </si>
+  <si>
+    <t>Excluded from model inputs; used for retrospective contact-efficiency analysis. Excluded from model inputs (final contact count is not known at the decision point). Kept in the full cleaned table for retrospective contacts-per-subscriber evaluation; removed from bank_marketing_model_inputs.csv.</t>
+  </si>
+  <si>
+    <t>previously_contacted</t>
+  </si>
+  <si>
+    <t>integer (0, 1)</t>
+  </si>
+  <si>
+    <t>1 if the customer had at least one contact before this campaign, else 0</t>
+  </si>
+  <si>
+    <t>1 = previous &gt; 0; 0 = previous = 0. Built from previous, not pdays, because 4,110 rows have pdays = 999 but a recorded earlier contact. No missing values.</t>
+  </si>
+  <si>
+    <t>Derived feature; model input</t>
+  </si>
+  <si>
+    <t>days_since_previous_contact</t>
+  </si>
+  <si>
+    <t>Days since the last contact in an earlier campaign</t>
+  </si>
+  <si>
+    <t>0 to 27 days. Missing (NaN) where pdays = 999 (39,673 rows). Never filled in the pipeline.</t>
+  </si>
+  <si>
+    <t>Derived feature; model input. Missing values handled in Module 4</t>
   </si>
 </sst>
 </file>
@@ -630,9 +657,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -645,9 +669,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -657,6 +678,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -992,7 +1019,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B842B66-B478-4078-BEC1-6CD4806E2082}">
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F73"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.90625" style="1" customWidth="1"/>
@@ -1013,14 +1040,14 @@
       <c r="F1" s="2"/>
     </row>
     <row r="2" spans="1:6" ht="20" x14ac:dyDescent="0.4">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -1031,7 +1058,7 @@
       <c r="F3" s="2"/>
     </row>
     <row r="4" spans="1:6" ht="15" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B4" s="2"/>
@@ -1041,10 +1068,10 @@
       <c r="F4" s="2"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="5" t="s">
         <v>3</v>
       </c>
       <c r="C5" s="2"/>
@@ -1053,10 +1080,10 @@
       <c r="F5" s="2"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="7" t="s">
         <v>5</v>
       </c>
       <c r="C6" s="2"/>
@@ -1065,10 +1092,10 @@
       <c r="F6" s="2"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C7" s="2"/>
@@ -1077,10 +1104,10 @@
       <c r="F7" s="2"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="7" t="s">
         <v>9</v>
       </c>
       <c r="C8" s="2"/>
@@ -1089,10 +1116,10 @@
       <c r="F8" s="2"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="7" t="s">
         <v>11</v>
       </c>
       <c r="C9" s="2"/>
@@ -1101,10 +1128,10 @@
       <c r="F9" s="2"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="7" t="s">
         <v>13</v>
       </c>
       <c r="C10" s="2"/>
@@ -1113,10 +1140,10 @@
       <c r="F10" s="2"/>
     </row>
     <row r="11" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="8" t="s">
         <v>15</v>
       </c>
       <c r="C11" s="2"/>
@@ -1125,10 +1152,10 @@
       <c r="F11" s="2"/>
     </row>
     <row r="12" spans="1:6" ht="28" x14ac:dyDescent="0.3">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="7" t="s">
         <v>17</v>
       </c>
       <c r="C12" s="2"/>
@@ -1137,10 +1164,10 @@
       <c r="F12" s="2"/>
     </row>
     <row r="13" spans="1:6" ht="28" x14ac:dyDescent="0.3">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="7" t="s">
         <v>19</v>
       </c>
       <c r="C13" s="2"/>
@@ -1149,10 +1176,10 @@
       <c r="F13" s="2"/>
     </row>
     <row r="14" spans="1:6" ht="29" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="8" t="s">
         <v>21</v>
       </c>
       <c r="C14" s="2"/>
@@ -1169,14 +1196,14 @@
       <c r="F15" s="2"/>
     </row>
     <row r="16" spans="1:6" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="10" t="s">
-        <v>166</v>
-      </c>
-      <c r="B16" s="10"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
+      <c r="A16" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="B16" s="14"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="2"/>
@@ -1187,7 +1214,7 @@
       <c r="F17" s="2"/>
     </row>
     <row r="18" spans="1:6" ht="15" x14ac:dyDescent="0.3">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="3" t="s">
         <v>22</v>
       </c>
       <c r="B18" s="2"/>
@@ -1197,7 +1224,7 @@
       <c r="F18" s="2"/>
     </row>
     <row r="19" spans="1:6" ht="15" x14ac:dyDescent="0.3">
-      <c r="A19" s="4"/>
+      <c r="A19" s="3"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
@@ -1205,7 +1232,7 @@
       <c r="F19" s="2"/>
     </row>
     <row r="20" spans="1:6" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B20" s="2"/>
@@ -1215,162 +1242,162 @@
       <c r="F20" s="2"/>
     </row>
     <row r="21" spans="1:6" ht="28" x14ac:dyDescent="0.3">
-      <c r="A21" s="11" t="s">
+      <c r="A21" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B21" s="11" t="s">
+      <c r="B21" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="D21" s="11" t="s">
+      <c r="D21" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="E21" s="11" t="s">
+      <c r="E21" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F21" s="11" t="s">
+      <c r="F21" s="9" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="42" x14ac:dyDescent="0.3">
-      <c r="A22" s="9" t="s">
+      <c r="A22" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B22" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="C22" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="D22" s="9" t="s">
+      <c r="D22" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="E22" s="9" t="s">
+      <c r="E22" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="F22" s="9" t="s">
+      <c r="F22" s="8" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="28" x14ac:dyDescent="0.3">
-      <c r="A23" s="9" t="s">
+      <c r="A23" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="B23" s="9" t="s">
+      <c r="B23" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="D23" s="9" t="s">
+      <c r="D23" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="E23" s="9" t="s">
+      <c r="E23" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="F23" s="9" t="s">
+      <c r="F23" s="8" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="28" x14ac:dyDescent="0.3">
-      <c r="A24" s="9" t="s">
+      <c r="A24" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="B24" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C24" s="9" t="s">
+      <c r="C24" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="D24" s="9" t="s">
+      <c r="D24" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="E24" s="9" t="s">
+      <c r="E24" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="F24" s="9" t="s">
+      <c r="F24" s="8" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="28" x14ac:dyDescent="0.3">
-      <c r="A25" s="9" t="s">
+      <c r="A25" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C25" s="9" t="s">
+      <c r="C25" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="D25" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="E25" s="9" t="s">
+      <c r="E25" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="F25" s="9" t="s">
+      <c r="F25" s="8" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="56" x14ac:dyDescent="0.3">
-      <c r="A26" s="9" t="s">
+      <c r="A26" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="B26" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="C26" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="D26" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="E26" s="9" t="s">
+      <c r="E26" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="F26" s="9" t="s">
+      <c r="F26" s="8" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="42" x14ac:dyDescent="0.3">
-      <c r="A27" s="9" t="s">
+    <row r="27" spans="1:6" ht="28" x14ac:dyDescent="0.3">
+      <c r="A27" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="B27" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="C27" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="D27" s="9" t="s">
+      <c r="D27" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="E27" s="9" t="s">
+      <c r="E27" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="F27" s="9" t="s">
+      <c r="F27" s="8" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="42" x14ac:dyDescent="0.3">
-      <c r="A28" s="9" t="s">
+    <row r="28" spans="1:6" ht="28" x14ac:dyDescent="0.3">
+      <c r="A28" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="B28" s="9" t="s">
+      <c r="B28" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C28" s="9" t="s">
+      <c r="C28" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="D28" s="9" t="s">
+      <c r="D28" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="E28" s="9" t="s">
+      <c r="E28" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="F28" s="9" t="s">
+      <c r="F28" s="8" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1383,7 +1410,7 @@
       <c r="F29" s="2"/>
     </row>
     <row r="30" spans="1:6" ht="15" x14ac:dyDescent="0.3">
-      <c r="A30" s="4" t="s">
+      <c r="A30" s="3" t="s">
         <v>58</v>
       </c>
       <c r="B30" s="2"/>
@@ -1393,143 +1420,143 @@
       <c r="F30" s="2"/>
     </row>
     <row r="31" spans="1:6" ht="28" x14ac:dyDescent="0.3">
-      <c r="A31" s="11" t="s">
+      <c r="A31" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B31" s="11" t="s">
+      <c r="B31" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C31" s="11" t="s">
+      <c r="C31" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="D31" s="11" t="s">
+      <c r="D31" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="E31" s="11" t="s">
+      <c r="E31" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F31" s="11" t="s">
+      <c r="F31" s="9" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="70" x14ac:dyDescent="0.3">
-      <c r="A32" s="9" t="s">
+      <c r="A32" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="B32" s="9" t="s">
+      <c r="B32" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C32" s="9" t="s">
+      <c r="C32" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="D32" s="9" t="s">
+      <c r="D32" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="E32" s="9" t="s">
+      <c r="E32" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="F32" s="9" t="s">
+      <c r="F32" s="8" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="70" x14ac:dyDescent="0.3">
-      <c r="A33" s="9" t="s">
+    <row r="33" spans="1:6" ht="56" x14ac:dyDescent="0.3">
+      <c r="A33" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="B33" s="9" t="s">
+      <c r="B33" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C33" s="9" t="s">
+      <c r="C33" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="D33" s="9" t="s">
+      <c r="D33" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="E33" s="9" t="s">
+      <c r="E33" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="F33" s="9" t="s">
+      <c r="F33" s="8" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="56" x14ac:dyDescent="0.3">
-      <c r="A34" s="9" t="s">
+      <c r="A34" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="B34" s="9" t="s">
+      <c r="B34" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C34" s="9" t="s">
+      <c r="C34" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="D34" s="9" t="s">
+      <c r="D34" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="E34" s="9" t="s">
+      <c r="E34" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="F34" s="9" t="s">
+      <c r="F34" s="8" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="56" x14ac:dyDescent="0.3">
-      <c r="A35" s="9" t="s">
+    <row r="35" spans="1:6" ht="196" x14ac:dyDescent="0.3">
+      <c r="A35" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="B35" s="9" t="s">
+      <c r="B35" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C35" s="9" t="s">
+      <c r="C35" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="D35" s="9" t="s">
+      <c r="D35" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="E35" s="9" t="s">
+      <c r="E35" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="F35" s="9" t="s">
+      <c r="F35" s="8" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="224" x14ac:dyDescent="0.3">
+      <c r="A36" s="8" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" ht="98" x14ac:dyDescent="0.3">
-      <c r="A36" s="9" t="s">
+      <c r="B36" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C36" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="B36" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C36" s="9" t="s">
+      <c r="D36" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="D36" s="9" t="s">
+      <c r="E36" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="E36" s="9" t="s">
+      <c r="F36" s="8" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="56" x14ac:dyDescent="0.3">
+      <c r="A37" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="F36" s="9" t="s">
+      <c r="B37" s="8" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" ht="84" x14ac:dyDescent="0.3">
-      <c r="A37" s="9" t="s">
+      <c r="C37" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="B37" s="9" t="s">
+      <c r="D37" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="C37" s="9" t="s">
+      <c r="E37" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="D37" s="9" t="s">
+      <c r="F37" s="8" t="s">
         <v>87</v>
-      </c>
-      <c r="E37" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="F37" s="9" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
@@ -1541,8 +1568,8 @@
       <c r="F38" s="2"/>
     </row>
     <row r="39" spans="1:6" ht="15" x14ac:dyDescent="0.3">
-      <c r="A39" s="4" t="s">
-        <v>90</v>
+      <c r="A39" s="3" t="s">
+        <v>88</v>
       </c>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
@@ -1551,477 +1578,517 @@
       <c r="F39" s="2"/>
     </row>
     <row r="40" spans="1:6" ht="28" x14ac:dyDescent="0.3">
-      <c r="A40" s="11" t="s">
+      <c r="A40" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B40" s="11" t="s">
+      <c r="B40" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C40" s="11" t="s">
+      <c r="C40" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="D40" s="11" t="s">
+      <c r="D40" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="E40" s="11" t="s">
+      <c r="E40" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F40" s="11" t="s">
+      <c r="F40" s="9" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="84" x14ac:dyDescent="0.3">
-      <c r="A41" s="9" t="s">
+    <row r="41" spans="1:6" ht="70" x14ac:dyDescent="0.3">
+      <c r="A41" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="B41" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C41" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="D41" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="B41" s="9" t="s">
+      <c r="E41" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="F41" s="8" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="56" x14ac:dyDescent="0.3">
+      <c r="A42" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="B42" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C41" s="9" t="s">
+      <c r="C42" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="D42" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="E42" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="D41" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="E41" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="F41" s="9" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="84" x14ac:dyDescent="0.3">
-      <c r="A42" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="B42" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C42" s="9" t="s">
+      <c r="F42" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="D42" s="9" t="s">
+    </row>
+    <row r="43" spans="1:6" ht="56" x14ac:dyDescent="0.3">
+      <c r="A43" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="E42" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="F42" s="9" t="s">
+      <c r="B43" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C43" s="8" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" ht="56" x14ac:dyDescent="0.3">
-      <c r="A43" s="9" t="s">
+      <c r="D43" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="B43" s="9" t="s">
+      <c r="E43" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="F43" s="8" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="98" x14ac:dyDescent="0.3">
+      <c r="A44" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="D44" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="E44" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F44" s="8" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="70" x14ac:dyDescent="0.3">
+      <c r="A45" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="B45" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="C45" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="D45" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="E45" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F45" s="8" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" s="2"/>
+      <c r="B46" s="2"/>
+      <c r="C46" s="2"/>
+      <c r="D46" s="2"/>
+      <c r="E46" s="2"/>
+      <c r="F46" s="2"/>
+    </row>
+    <row r="47" spans="1:6" ht="15" x14ac:dyDescent="0.3">
+      <c r="A47" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="2"/>
+      <c r="F47" s="2"/>
+    </row>
+    <row r="48" spans="1:6" ht="28" x14ac:dyDescent="0.3">
+      <c r="A48" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F48" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="70" x14ac:dyDescent="0.3">
+      <c r="A49" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B49" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="C49" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="D49" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="E49" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="F49" s="8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="56" x14ac:dyDescent="0.3">
+      <c r="A50" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B50" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="D50" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="E50" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="F50" s="8" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" ht="42" x14ac:dyDescent="0.3">
+      <c r="A51" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="B51" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="C51" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="D51" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="E51" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="F51" s="8" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" ht="56" x14ac:dyDescent="0.3">
+      <c r="A52" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B52" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="C52" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="D52" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="E52" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="F52" s="8" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="70" x14ac:dyDescent="0.3">
+      <c r="A53" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="B53" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="C53" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="D53" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="E53" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="F53" s="8" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A54" s="2"/>
+      <c r="B54" s="2"/>
+      <c r="C54" s="2"/>
+      <c r="D54" s="2"/>
+      <c r="E54" s="2"/>
+      <c r="F54" s="2"/>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A55" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="B55" s="2"/>
+      <c r="C55" s="2"/>
+      <c r="D55" s="2"/>
+      <c r="E55" s="2"/>
+      <c r="F55" s="2"/>
+    </row>
+    <row r="56" spans="1:6" ht="28" x14ac:dyDescent="0.3">
+      <c r="A56" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B56" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C56" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D56" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E56" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F56" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" ht="56" x14ac:dyDescent="0.3">
+      <c r="A57" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="B57" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C43" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="D43" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="E43" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="F43" s="9" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A44" s="2"/>
-      <c r="B44" s="2"/>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
-      <c r="E44" s="2"/>
-      <c r="F44" s="2"/>
-    </row>
-    <row r="45" spans="1:6" ht="15" x14ac:dyDescent="0.3">
-      <c r="A45" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
-      <c r="F45" s="2"/>
-    </row>
-    <row r="46" spans="1:6" ht="28" x14ac:dyDescent="0.3">
-      <c r="A46" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B46" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C46" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="D46" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="F46" s="6" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" ht="70" x14ac:dyDescent="0.3">
-      <c r="A47" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="B47" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="C47" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="D47" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="E47" s="9" t="s">
-        <v>109</v>
-      </c>
-      <c r="F47" s="9" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" ht="56" x14ac:dyDescent="0.3">
-      <c r="A48" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="B48" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="C48" s="9" t="s">
-        <v>112</v>
-      </c>
-      <c r="D48" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="E48" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="F48" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" ht="42" x14ac:dyDescent="0.3">
-      <c r="A49" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="B49" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="C49" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="D49" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="E49" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="F49" s="9" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" ht="56" x14ac:dyDescent="0.3">
-      <c r="A50" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="B50" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="C50" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="D50" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="E50" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="F50" s="9" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" ht="84" x14ac:dyDescent="0.3">
-      <c r="A51" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="B51" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="C51" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="D51" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="E51" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="F51" s="9" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A52" s="2"/>
-      <c r="B52" s="2"/>
-      <c r="C52" s="2"/>
-      <c r="D52" s="2"/>
-      <c r="E52" s="2"/>
-      <c r="F52" s="2"/>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53" s="12" t="s">
+      <c r="C57" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="B53" s="2"/>
-      <c r="C53" s="2"/>
-      <c r="D53" s="2"/>
-      <c r="E53" s="2"/>
-      <c r="F53" s="2"/>
-    </row>
-    <row r="54" spans="1:6" ht="28" x14ac:dyDescent="0.3">
-      <c r="A54" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B54" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="D54" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="E54" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="F54" s="6" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" ht="56" x14ac:dyDescent="0.3">
-      <c r="A55" s="9" t="s">
+      <c r="D57" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="B55" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="C55" s="9" t="s">
+      <c r="E57" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="D55" s="9" t="s">
+      <c r="F57" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="E55" s="9" t="s">
-        <v>133</v>
-      </c>
-      <c r="F55" s="9" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56" s="2"/>
-      <c r="B56" s="2"/>
-      <c r="C56" s="2"/>
-      <c r="D56" s="2"/>
-      <c r="E56" s="2"/>
-      <c r="F56" s="2"/>
-    </row>
-    <row r="57" spans="1:6" ht="15" x14ac:dyDescent="0.3">
-      <c r="A57" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="B57" s="2"/>
-      <c r="C57" s="2"/>
-      <c r="D57" s="2"/>
-      <c r="E57" s="2"/>
-      <c r="F57" s="2"/>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="2" t="s">
-        <v>136</v>
-      </c>
+      <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
       <c r="D58" s="2"/>
       <c r="E58" s="2"/>
       <c r="F58" s="2"/>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A59" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="B59" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="C59" s="6" t="s">
-        <v>139</v>
-      </c>
+    <row r="59" spans="1:6" ht="15" x14ac:dyDescent="0.3">
+      <c r="A59" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B59" s="2"/>
+      <c r="C59" s="2"/>
       <c r="D59" s="2"/>
       <c r="E59" s="2"/>
       <c r="F59" s="2"/>
     </row>
-    <row r="60" spans="1:6" ht="28" x14ac:dyDescent="0.3">
-      <c r="A60" s="9" t="s">
-        <v>140</v>
-      </c>
-      <c r="B60" s="9" t="s">
-        <v>141</v>
-      </c>
-      <c r="C60" s="9" t="s">
-        <v>142</v>
-      </c>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A60" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B60" s="2"/>
+      <c r="C60" s="2"/>
       <c r="D60" s="2"/>
       <c r="E60" s="2"/>
       <c r="F60" s="2"/>
     </row>
-    <row r="61" spans="1:6" ht="42" x14ac:dyDescent="0.3">
-      <c r="A61" s="9" t="s">
-        <v>143</v>
-      </c>
-      <c r="B61" s="9" t="s">
-        <v>144</v>
-      </c>
-      <c r="C61" s="9" t="s">
-        <v>145</v>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A61" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="B61" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C61" s="5" t="s">
+        <v>137</v>
       </c>
       <c r="D61" s="2"/>
       <c r="E61" s="2"/>
       <c r="F61" s="2"/>
     </row>
     <row r="62" spans="1:6" ht="28" x14ac:dyDescent="0.3">
-      <c r="A62" s="9" t="s">
-        <v>146</v>
-      </c>
-      <c r="B62" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="C62" s="9" t="s">
-        <v>148</v>
+      <c r="A62" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="B62" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="C62" s="8" t="s">
+        <v>140</v>
       </c>
       <c r="D62" s="2"/>
       <c r="E62" s="2"/>
       <c r="F62" s="2"/>
     </row>
-    <row r="63" spans="1:6" ht="70" x14ac:dyDescent="0.3">
-      <c r="A63" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="B63" s="9" t="s">
-        <v>150</v>
-      </c>
-      <c r="C63" s="9" t="s">
-        <v>151</v>
+    <row r="63" spans="1:6" ht="42" x14ac:dyDescent="0.3">
+      <c r="A63" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="B63" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="C63" s="8" t="s">
+        <v>143</v>
       </c>
       <c r="D63" s="2"/>
       <c r="E63" s="2"/>
       <c r="F63" s="2"/>
     </row>
-    <row r="64" spans="1:6" ht="56" x14ac:dyDescent="0.3">
-      <c r="A64" s="9" t="s">
-        <v>152</v>
-      </c>
-      <c r="B64" s="9" t="s">
-        <v>153</v>
-      </c>
-      <c r="C64" s="9" t="s">
-        <v>154</v>
+    <row r="64" spans="1:6" ht="28" x14ac:dyDescent="0.3">
+      <c r="A64" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="B64" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="C64" s="8" t="s">
+        <v>146</v>
       </c>
       <c r="D64" s="2"/>
       <c r="E64" s="2"/>
       <c r="F64" s="2"/>
     </row>
-    <row r="65" spans="1:6" ht="42" x14ac:dyDescent="0.3">
-      <c r="A65" s="9" t="s">
-        <v>155</v>
-      </c>
-      <c r="B65" s="9" t="s">
-        <v>156</v>
-      </c>
-      <c r="C65" s="9" t="s">
-        <v>157</v>
+    <row r="65" spans="1:6" ht="70" x14ac:dyDescent="0.3">
+      <c r="A65" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="B65" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="C65" s="8" t="s">
+        <v>149</v>
       </c>
       <c r="D65" s="2"/>
       <c r="E65" s="2"/>
       <c r="F65" s="2"/>
     </row>
-    <row r="66" spans="1:6" ht="112" x14ac:dyDescent="0.3">
-      <c r="A66" s="9" t="s">
-        <v>158</v>
-      </c>
-      <c r="B66" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="C66" s="9" t="s">
-        <v>160</v>
+    <row r="66" spans="1:6" ht="56" x14ac:dyDescent="0.3">
+      <c r="A66" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="B66" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="C66" s="8" t="s">
+        <v>152</v>
       </c>
       <c r="D66" s="2"/>
       <c r="E66" s="2"/>
       <c r="F66" s="2"/>
     </row>
-    <row r="67" spans="1:6" ht="56" x14ac:dyDescent="0.3">
-      <c r="A67" s="9" t="s">
-        <v>161</v>
-      </c>
-      <c r="B67" s="9" t="s">
-        <v>162</v>
-      </c>
-      <c r="C67" s="9" t="s">
-        <v>163</v>
+    <row r="67" spans="1:6" ht="42" x14ac:dyDescent="0.3">
+      <c r="A67" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="B67" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="C67" s="8" t="s">
+        <v>155</v>
       </c>
       <c r="D67" s="2"/>
       <c r="E67" s="2"/>
       <c r="F67" s="2"/>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A68" s="13" t="s">
-        <v>164</v>
-      </c>
-      <c r="B68" s="13"/>
-      <c r="C68" s="13"/>
-      <c r="D68" s="13"/>
-      <c r="E68" s="13"/>
-      <c r="F68" s="13"/>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A69" s="2"/>
-      <c r="B69" s="2"/>
-      <c r="C69" s="2"/>
+    <row r="68" spans="1:6" ht="112" x14ac:dyDescent="0.3">
+      <c r="A68" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="B68" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="C68" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="D68" s="2"/>
+      <c r="E68" s="2"/>
+      <c r="F68" s="2"/>
+    </row>
+    <row r="69" spans="1:6" ht="56" x14ac:dyDescent="0.3">
+      <c r="A69" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="B69" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="C69" s="8" t="s">
+        <v>161</v>
+      </c>
       <c r="D69" s="2"/>
       <c r="E69" s="2"/>
       <c r="F69" s="2"/>
     </row>
-    <row r="70" spans="1:6" ht="15" x14ac:dyDescent="0.3">
-      <c r="A70" s="4" t="s">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A70" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="B70" s="11"/>
+      <c r="C70" s="11"/>
+      <c r="D70" s="11"/>
+      <c r="E70" s="11"/>
+      <c r="F70" s="11"/>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A71" s="2"/>
+      <c r="B71" s="2"/>
+      <c r="C71" s="2"/>
+      <c r="D71" s="2"/>
+      <c r="E71" s="2"/>
+      <c r="F71" s="2"/>
+    </row>
+    <row r="72" spans="1:6" ht="15" x14ac:dyDescent="0.3">
+      <c r="A72" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B72" s="2"/>
+      <c r="C72" s="2"/>
+      <c r="D72" s="2"/>
+      <c r="E72" s="2"/>
+      <c r="F72" s="2"/>
+    </row>
+    <row r="73" spans="1:6" ht="134.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="B70" s="2"/>
-      <c r="C70" s="2"/>
-      <c r="D70" s="2"/>
-      <c r="E70" s="2"/>
-      <c r="F70" s="2"/>
-    </row>
-    <row r="71" spans="1:6" ht="134.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="14" t="s">
-        <v>167</v>
-      </c>
-      <c r="B71" s="14"/>
-      <c r="C71" s="14"/>
-      <c r="D71" s="14"/>
-      <c r="E71" s="14"/>
-      <c r="F71" s="14"/>
+      <c r="B73" s="12"/>
+      <c r="C73" s="12"/>
+      <c r="D73" s="12"/>
+      <c r="E73" s="12"/>
+      <c r="F73" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A68:F68"/>
-    <mergeCell ref="A71:F71"/>
+    <mergeCell ref="A70:F70"/>
+    <mergeCell ref="A73:F73"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A16:F16"/>
   </mergeCells>

</xml_diff>